<commit_message>
Changes, & Bug Fixing 9
</commit_message>
<xml_diff>
--- a/public/downloads/Portal_Features_Catalog.xlsx
+++ b/public/downloads/Portal_Features_Catalog.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Features Catalog" sheetId="1" r:id="rId4"/>
     <sheet name="ROI &amp; Impact Analysis" sheetId="2" r:id="rId5"/>
-    <sheet name="Commercial Proposal" sheetId="3" r:id="rId6"/>
+    <sheet name="Implementation Roadmap" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="245">
   <si>
     <t>SMART BLOOD BANK &amp; DONOR MANAGEMENT PORTAL - FEATURE CATALOG</t>
   </si>
@@ -661,82 +661,97 @@
     <t>Provides 100% accurate data for foreign grants and audits</t>
   </si>
   <si>
-    <t>COMMERCIAL LICENSING &amp; IMPLEMENTATION PROPOSAL</t>
-  </si>
-  <si>
-    <t>Package Tier</t>
-  </si>
-  <si>
-    <t>Target Organization</t>
-  </si>
-  <si>
-    <t>Initial Asking Price (PKR)</t>
-  </si>
-  <si>
-    <t>Negotiated Target (PKR)</t>
-  </si>
-  <si>
-    <t>Scope of Features &amp; Support</t>
-  </si>
-  <si>
-    <t>Starter NGO Edition</t>
-  </si>
-  <si>
-    <t>Local City Trusts, Small Welfare Societies</t>
-  </si>
-  <si>
-    <t>Rs. 180,000 - 250,000</t>
-  </si>
-  <si>
-    <t>Rs. 120,000 - 150,000</t>
-  </si>
-  <si>
-    <t>Core Donor Registry, Cooldown Countdown, Emergency Matching, Free 1-Click WhatsApp, Basic Reports, 3 Staff Users, 30-Day Support</t>
-  </si>
-  <si>
-    <t>Professional Center Edition (Recommended)</t>
-  </si>
-  <si>
-    <t>Established Thalassemia Centers, Regional Hospitals, Welfare Foundations</t>
-  </si>
-  <si>
-    <t>Rs. 350,000 - 450,000</t>
-  </si>
-  <si>
-    <t>Rs. 250,000 - 300,000</t>
-  </si>
-  <si>
-    <t>All Starter Features + Digital QR Verified Donor Cards, Public Emergency Request Portal, Gamification Badges, Official PDF Certificates, Full Urdu RTL + English, Dark Mode, Bulk CSV Import/Export, Unlimited Users, 90-Day Priority Support</t>
-  </si>
-  <si>
-    <t>Enterprise Network License</t>
-  </si>
-  <si>
-    <t>Nationwide Trusts, Multi-Branch Foundations, Government Partners</t>
-  </si>
-  <si>
-    <t>Rs. 600,000 - 800,000+</t>
-  </si>
-  <si>
-    <t>Rs. 450,000 - 550,000</t>
-  </si>
-  <si>
-    <t>All Professional Features + Multi-Branch Architecture, Custom Hospital ERP Integration, Dedicated Cloud Server &amp; SSL Setup, White-Label Domain &amp; Branding, 1 Year Annual Maintenance Contract (AMC), 24/7 Priority SLA</t>
-  </si>
-  <si>
-    <t>Annual Maintenance Contract (AMC)</t>
-  </si>
-  <si>
-    <t>Ongoing Server Maintenance, Backups &amp; Technical Support</t>
-  </si>
-  <si>
-    <t>Rs. 15,000 / month</t>
-  </si>
-  <si>
-    <t>Rs. 10,000 - 12,000 / month</t>
-  </si>
-  <si>
-    <t>24/7 Server monitoring, automated database backups, security patches, minor UI tweaks, and staff support.</t>
+    <t>14-DAY IMPLEMENTATION ROADMAP &amp; DATA GOVERNANCE</t>
+  </si>
+  <si>
+    <t>Phase #</t>
+  </si>
+  <si>
+    <t>Timeline</t>
+  </si>
+  <si>
+    <t>Phase Title</t>
+  </si>
+  <si>
+    <t>Core Deliverables</t>
+  </si>
+  <si>
+    <t>Responsible Stakeholders</t>
+  </si>
+  <si>
+    <t>Phase 01</t>
+  </si>
+  <si>
+    <t>Days 1 – 3</t>
+  </si>
+  <si>
+    <t>Cloud Infrastructure &amp; Custom Branding</t>
+  </si>
+  <si>
+    <t>Dedicated server provisioning, SSL certificate installation, domain binding, NGO logo/color configuration.</t>
+  </si>
+  <si>
+    <t>IT Lead &amp; DevOps</t>
+  </si>
+  <si>
+    <t>Phase 02</t>
+  </si>
+  <si>
+    <t>Days 4 – 7</t>
+  </si>
+  <si>
+    <t>Historical Data Cleansing &amp; CSV Migration</t>
+  </si>
+  <si>
+    <t>Sanitizing legacy donor records, duplicate removal, bulk CSV import, and unique registration ID generation.</t>
+  </si>
+  <si>
+    <t>Data Specialist &amp; Admin</t>
+  </si>
+  <si>
+    <t>Phase 03</t>
+  </si>
+  <si>
+    <t>Days 8 – 11</t>
+  </si>
+  <si>
+    <t>Staff Training &amp; Role-Based Access Setup</t>
+  </si>
+  <si>
+    <t>Role configuration (Spatie RBAC), coordinator training for emergency dispatch and WhatsApp, doctor walkthrough.</t>
+  </si>
+  <si>
+    <t>Lead Trainer &amp; Medical Staff</t>
+  </si>
+  <si>
+    <t>Phase 04</t>
+  </si>
+  <si>
+    <t>Days 12 – 14</t>
+  </si>
+  <si>
+    <t>Pilot Verification &amp; Official Go-Live</t>
+  </si>
+  <si>
+    <t>Live QR code mobile scanning tests with partner hospitals, emergency public portal activation, helpline launch.</t>
+  </si>
+  <si>
+    <t>Executive Director &amp; Operations</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
+  </si>
+  <si>
+    <t>Post Go-Live</t>
+  </si>
+  <si>
+    <t>Security Governance &amp; System Monitoring</t>
+  </si>
+  <si>
+    <t>Automated daily database backups, HIPAA-aligned donor privacy, 24/7 server health tracking, and continuous upgrades.</t>
+  </si>
+  <si>
+    <t>SLA Support &amp; Systems Lead</t>
   </si>
 </sst>
 </file>
@@ -744,7 +759,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -805,11 +820,20 @@
       <strike val="0"/>
       <u val="none"/>
       <sz val="11"/>
+      <color rgb="FF059669"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -843,12 +867,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1565A8"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -895,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -935,11 +953,9 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="7" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="6" numFmtId="0" fillId="5" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="7" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="7" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="7" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="7" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="7" numFmtId="0" fillId="5" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2320,14 +2336,14 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="49.417" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="85.979" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="33.992" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="32.992" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="280.646" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="49.417" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="137.966" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="37.705" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" customHeight="1" ht="40">
@@ -2356,13 +2372,13 @@
       <c r="A3" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="5" t="s">
         <v>223</v>
       </c>
       <c r="E3" s="5" t="s">
@@ -2373,16 +2389,16 @@
       <c r="A4" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="4" t="s">
         <v>229</v>
       </c>
     </row>
@@ -2390,13 +2406,13 @@
       <c r="A5" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="5" t="s">
         <v>233</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -2404,20 +2420,37 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="16" t="s">
         <v>236</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="4" t="s">
         <v>238</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>239</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>